<commit_message>
Jour 22 : Power Query avancé
</commit_message>
<xml_diff>
--- a/jour-21-power-query/data/ventes.xlsx
+++ b/jour-21-power-query/data/ventes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdou\OneDrive\Documents\BootcampExcel\excel-bootcamp-30-jours\jour-21-power-query\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAF750E-FC43-4237-9442-4741A22FFE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34D3CDA5-97EF-4F1D-AB47-AF42ABD782F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{5B6C3E0D-B841-4927-BA65-739CCD248B7F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="220">
   <si>
     <t>Vente_ID</t>
   </si>
@@ -396,6 +396,306 @@
   </si>
   <si>
     <t>V100</t>
+  </si>
+  <si>
+    <t>V101</t>
+  </si>
+  <si>
+    <t>V102</t>
+  </si>
+  <si>
+    <t>V103</t>
+  </si>
+  <si>
+    <t>V104</t>
+  </si>
+  <si>
+    <t>V105</t>
+  </si>
+  <si>
+    <t>V106</t>
+  </si>
+  <si>
+    <t>V107</t>
+  </si>
+  <si>
+    <t>V108</t>
+  </si>
+  <si>
+    <t>V109</t>
+  </si>
+  <si>
+    <t>V110</t>
+  </si>
+  <si>
+    <t>V111</t>
+  </si>
+  <si>
+    <t>V112</t>
+  </si>
+  <si>
+    <t>V113</t>
+  </si>
+  <si>
+    <t>V114</t>
+  </si>
+  <si>
+    <t>V115</t>
+  </si>
+  <si>
+    <t>V116</t>
+  </si>
+  <si>
+    <t>V117</t>
+  </si>
+  <si>
+    <t>V118</t>
+  </si>
+  <si>
+    <t>V119</t>
+  </si>
+  <si>
+    <t>V120</t>
+  </si>
+  <si>
+    <t>V121</t>
+  </si>
+  <si>
+    <t>V122</t>
+  </si>
+  <si>
+    <t>V123</t>
+  </si>
+  <si>
+    <t>V124</t>
+  </si>
+  <si>
+    <t>V125</t>
+  </si>
+  <si>
+    <t>V126</t>
+  </si>
+  <si>
+    <t>V127</t>
+  </si>
+  <si>
+    <t>V128</t>
+  </si>
+  <si>
+    <t>V129</t>
+  </si>
+  <si>
+    <t>V130</t>
+  </si>
+  <si>
+    <t>V131</t>
+  </si>
+  <si>
+    <t>V132</t>
+  </si>
+  <si>
+    <t>V133</t>
+  </si>
+  <si>
+    <t>V134</t>
+  </si>
+  <si>
+    <t>V135</t>
+  </si>
+  <si>
+    <t>V136</t>
+  </si>
+  <si>
+    <t>V137</t>
+  </si>
+  <si>
+    <t>V138</t>
+  </si>
+  <si>
+    <t>V139</t>
+  </si>
+  <si>
+    <t>V140</t>
+  </si>
+  <si>
+    <t>V141</t>
+  </si>
+  <si>
+    <t>V142</t>
+  </si>
+  <si>
+    <t>V143</t>
+  </si>
+  <si>
+    <t>V144</t>
+  </si>
+  <si>
+    <t>V145</t>
+  </si>
+  <si>
+    <t>V146</t>
+  </si>
+  <si>
+    <t>V147</t>
+  </si>
+  <si>
+    <t>V148</t>
+  </si>
+  <si>
+    <t>V149</t>
+  </si>
+  <si>
+    <t>V150</t>
+  </si>
+  <si>
+    <t>V151</t>
+  </si>
+  <si>
+    <t>V152</t>
+  </si>
+  <si>
+    <t>V153</t>
+  </si>
+  <si>
+    <t>V154</t>
+  </si>
+  <si>
+    <t>V155</t>
+  </si>
+  <si>
+    <t>V156</t>
+  </si>
+  <si>
+    <t>V157</t>
+  </si>
+  <si>
+    <t>V158</t>
+  </si>
+  <si>
+    <t>V159</t>
+  </si>
+  <si>
+    <t>V160</t>
+  </si>
+  <si>
+    <t>V161</t>
+  </si>
+  <si>
+    <t>V162</t>
+  </si>
+  <si>
+    <t>V163</t>
+  </si>
+  <si>
+    <t>V164</t>
+  </si>
+  <si>
+    <t>V165</t>
+  </si>
+  <si>
+    <t>V166</t>
+  </si>
+  <si>
+    <t>V167</t>
+  </si>
+  <si>
+    <t>V168</t>
+  </si>
+  <si>
+    <t>V169</t>
+  </si>
+  <si>
+    <t>V170</t>
+  </si>
+  <si>
+    <t>V171</t>
+  </si>
+  <si>
+    <t>V172</t>
+  </si>
+  <si>
+    <t>V173</t>
+  </si>
+  <si>
+    <t>V174</t>
+  </si>
+  <si>
+    <t>V175</t>
+  </si>
+  <si>
+    <t>V176</t>
+  </si>
+  <si>
+    <t>V177</t>
+  </si>
+  <si>
+    <t>V178</t>
+  </si>
+  <si>
+    <t>V179</t>
+  </si>
+  <si>
+    <t>V180</t>
+  </si>
+  <si>
+    <t>V181</t>
+  </si>
+  <si>
+    <t>V182</t>
+  </si>
+  <si>
+    <t>V183</t>
+  </si>
+  <si>
+    <t>V184</t>
+  </si>
+  <si>
+    <t>V185</t>
+  </si>
+  <si>
+    <t>V186</t>
+  </si>
+  <si>
+    <t>V187</t>
+  </si>
+  <si>
+    <t>V188</t>
+  </si>
+  <si>
+    <t>V189</t>
+  </si>
+  <si>
+    <t>V190</t>
+  </si>
+  <si>
+    <t>V191</t>
+  </si>
+  <si>
+    <t>V192</t>
+  </si>
+  <si>
+    <t>V193</t>
+  </si>
+  <si>
+    <t>V194</t>
+  </si>
+  <si>
+    <t>V195</t>
+  </si>
+  <si>
+    <t>V196</t>
+  </si>
+  <si>
+    <t>V197</t>
+  </si>
+  <si>
+    <t>V198</t>
+  </si>
+  <si>
+    <t>V199</t>
+  </si>
+  <si>
+    <t>V200</t>
   </si>
 </sst>
 </file>
@@ -768,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E3FE89-8595-48DB-9DA5-5875CE08D2D8}">
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -2488,6 +2788,1706 @@
         <v>5</v>
       </c>
     </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A102" t="s">
+        <v>120</v>
+      </c>
+      <c r="B102" s="1">
+        <v>46143</v>
+      </c>
+      <c r="C102" t="s">
+        <v>6</v>
+      </c>
+      <c r="D102" t="s">
+        <v>7</v>
+      </c>
+      <c r="E102">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A103" t="s">
+        <v>121</v>
+      </c>
+      <c r="B103" s="1">
+        <v>46144</v>
+      </c>
+      <c r="C103" t="s">
+        <v>9</v>
+      </c>
+      <c r="D103" t="s">
+        <v>10</v>
+      </c>
+      <c r="E103">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A104" t="s">
+        <v>122</v>
+      </c>
+      <c r="B104" s="1">
+        <v>46145</v>
+      </c>
+      <c r="C104" t="s">
+        <v>70</v>
+      </c>
+      <c r="D104" t="s">
+        <v>15</v>
+      </c>
+      <c r="E104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A105" t="s">
+        <v>123</v>
+      </c>
+      <c r="B105" s="1">
+        <v>46146</v>
+      </c>
+      <c r="C105" t="s">
+        <v>12</v>
+      </c>
+      <c r="D105" t="s">
+        <v>7</v>
+      </c>
+      <c r="E105">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A106" t="s">
+        <v>124</v>
+      </c>
+      <c r="B106" s="1">
+        <v>46147</v>
+      </c>
+      <c r="C106" t="s">
+        <v>60</v>
+      </c>
+      <c r="D106" t="s">
+        <v>31</v>
+      </c>
+      <c r="E106">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A107" t="s">
+        <v>125</v>
+      </c>
+      <c r="B107" s="1">
+        <v>46148</v>
+      </c>
+      <c r="C107" t="s">
+        <v>6</v>
+      </c>
+      <c r="D107" t="s">
+        <v>17</v>
+      </c>
+      <c r="E107">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A108" t="s">
+        <v>126</v>
+      </c>
+      <c r="B108" s="1">
+        <v>46149</v>
+      </c>
+      <c r="C108" t="s">
+        <v>23</v>
+      </c>
+      <c r="D108" t="s">
+        <v>10</v>
+      </c>
+      <c r="E108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A109" t="s">
+        <v>127</v>
+      </c>
+      <c r="B109" s="1">
+        <v>46150</v>
+      </c>
+      <c r="C109" t="s">
+        <v>19</v>
+      </c>
+      <c r="D109" t="s">
+        <v>15</v>
+      </c>
+      <c r="E109">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A110" t="s">
+        <v>128</v>
+      </c>
+      <c r="B110" s="1">
+        <v>46151</v>
+      </c>
+      <c r="C110" t="s">
+        <v>65</v>
+      </c>
+      <c r="D110" t="s">
+        <v>7</v>
+      </c>
+      <c r="E110">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A111" t="s">
+        <v>129</v>
+      </c>
+      <c r="B111" s="1">
+        <v>46152</v>
+      </c>
+      <c r="C111" t="s">
+        <v>42</v>
+      </c>
+      <c r="D111" t="s">
+        <v>31</v>
+      </c>
+      <c r="E111">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A112" t="s">
+        <v>130</v>
+      </c>
+      <c r="B112" s="1">
+        <v>46153</v>
+      </c>
+      <c r="C112" t="s">
+        <v>9</v>
+      </c>
+      <c r="D112" t="s">
+        <v>10</v>
+      </c>
+      <c r="E112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A113" t="s">
+        <v>131</v>
+      </c>
+      <c r="B113" s="1">
+        <v>46154</v>
+      </c>
+      <c r="C113" t="s">
+        <v>21</v>
+      </c>
+      <c r="D113" t="s">
+        <v>17</v>
+      </c>
+      <c r="E113">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A114" t="s">
+        <v>132</v>
+      </c>
+      <c r="B114" s="1">
+        <v>46155</v>
+      </c>
+      <c r="C114" t="s">
+        <v>6</v>
+      </c>
+      <c r="D114" t="s">
+        <v>15</v>
+      </c>
+      <c r="E114">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A115" t="s">
+        <v>133</v>
+      </c>
+      <c r="B115" s="1">
+        <v>46156</v>
+      </c>
+      <c r="C115" t="s">
+        <v>70</v>
+      </c>
+      <c r="D115" t="s">
+        <v>7</v>
+      </c>
+      <c r="E115">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A116" t="s">
+        <v>134</v>
+      </c>
+      <c r="B116" s="1">
+        <v>46157</v>
+      </c>
+      <c r="C116" t="s">
+        <v>12</v>
+      </c>
+      <c r="D116" t="s">
+        <v>31</v>
+      </c>
+      <c r="E116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A117" t="s">
+        <v>135</v>
+      </c>
+      <c r="B117" s="1">
+        <v>46158</v>
+      </c>
+      <c r="C117" t="s">
+        <v>60</v>
+      </c>
+      <c r="D117" t="s">
+        <v>10</v>
+      </c>
+      <c r="E117">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A118" t="s">
+        <v>136</v>
+      </c>
+      <c r="B118" s="1">
+        <v>46159</v>
+      </c>
+      <c r="C118" t="s">
+        <v>65</v>
+      </c>
+      <c r="D118" t="s">
+        <v>17</v>
+      </c>
+      <c r="E118">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A119" t="s">
+        <v>137</v>
+      </c>
+      <c r="B119" s="1">
+        <v>46160</v>
+      </c>
+      <c r="C119" t="s">
+        <v>23</v>
+      </c>
+      <c r="D119" t="s">
+        <v>7</v>
+      </c>
+      <c r="E119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A120" t="s">
+        <v>138</v>
+      </c>
+      <c r="B120" s="1">
+        <v>46161</v>
+      </c>
+      <c r="C120" t="s">
+        <v>19</v>
+      </c>
+      <c r="D120" t="s">
+        <v>15</v>
+      </c>
+      <c r="E120">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A121" t="s">
+        <v>139</v>
+      </c>
+      <c r="B121" s="1">
+        <v>46162</v>
+      </c>
+      <c r="C121" t="s">
+        <v>42</v>
+      </c>
+      <c r="D121" t="s">
+        <v>10</v>
+      </c>
+      <c r="E121">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A122" t="s">
+        <v>140</v>
+      </c>
+      <c r="B122" s="1">
+        <v>46163</v>
+      </c>
+      <c r="C122" t="s">
+        <v>6</v>
+      </c>
+      <c r="D122" t="s">
+        <v>31</v>
+      </c>
+      <c r="E122">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A123" t="s">
+        <v>141</v>
+      </c>
+      <c r="B123" s="1">
+        <v>46164</v>
+      </c>
+      <c r="C123" t="s">
+        <v>21</v>
+      </c>
+      <c r="D123" t="s">
+        <v>7</v>
+      </c>
+      <c r="E123">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A124" t="s">
+        <v>142</v>
+      </c>
+      <c r="B124" s="1">
+        <v>46165</v>
+      </c>
+      <c r="C124" t="s">
+        <v>9</v>
+      </c>
+      <c r="D124" t="s">
+        <v>17</v>
+      </c>
+      <c r="E124">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A125" t="s">
+        <v>143</v>
+      </c>
+      <c r="B125" s="1">
+        <v>46166</v>
+      </c>
+      <c r="C125" t="s">
+        <v>70</v>
+      </c>
+      <c r="D125" t="s">
+        <v>10</v>
+      </c>
+      <c r="E125">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A126" t="s">
+        <v>144</v>
+      </c>
+      <c r="B126" s="1">
+        <v>46167</v>
+      </c>
+      <c r="C126" t="s">
+        <v>60</v>
+      </c>
+      <c r="D126" t="s">
+        <v>15</v>
+      </c>
+      <c r="E126">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A127" t="s">
+        <v>145</v>
+      </c>
+      <c r="B127" s="1">
+        <v>46168</v>
+      </c>
+      <c r="C127" t="s">
+        <v>12</v>
+      </c>
+      <c r="D127" t="s">
+        <v>7</v>
+      </c>
+      <c r="E127">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A128" t="s">
+        <v>146</v>
+      </c>
+      <c r="B128" s="1">
+        <v>46169</v>
+      </c>
+      <c r="C128" t="s">
+        <v>23</v>
+      </c>
+      <c r="D128" t="s">
+        <v>31</v>
+      </c>
+      <c r="E128">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A129" t="s">
+        <v>147</v>
+      </c>
+      <c r="B129" s="1">
+        <v>46170</v>
+      </c>
+      <c r="C129" t="s">
+        <v>65</v>
+      </c>
+      <c r="D129" t="s">
+        <v>17</v>
+      </c>
+      <c r="E129">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A130" t="s">
+        <v>148</v>
+      </c>
+      <c r="B130" s="1">
+        <v>46171</v>
+      </c>
+      <c r="C130" t="s">
+        <v>6</v>
+      </c>
+      <c r="D130" t="s">
+        <v>10</v>
+      </c>
+      <c r="E130">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A131" t="s">
+        <v>149</v>
+      </c>
+      <c r="B131" s="1">
+        <v>46172</v>
+      </c>
+      <c r="C131" t="s">
+        <v>19</v>
+      </c>
+      <c r="D131" t="s">
+        <v>15</v>
+      </c>
+      <c r="E131">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A132" t="s">
+        <v>150</v>
+      </c>
+      <c r="B132" s="1">
+        <v>46173</v>
+      </c>
+      <c r="C132" t="s">
+        <v>42</v>
+      </c>
+      <c r="D132" t="s">
+        <v>7</v>
+      </c>
+      <c r="E132">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A133" t="s">
+        <v>151</v>
+      </c>
+      <c r="B133" s="1">
+        <v>46174</v>
+      </c>
+      <c r="C133" t="s">
+        <v>9</v>
+      </c>
+      <c r="D133" t="s">
+        <v>31</v>
+      </c>
+      <c r="E133">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A134" t="s">
+        <v>152</v>
+      </c>
+      <c r="B134" s="1">
+        <v>46175</v>
+      </c>
+      <c r="C134" t="s">
+        <v>21</v>
+      </c>
+      <c r="D134" t="s">
+        <v>17</v>
+      </c>
+      <c r="E134">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A135" t="s">
+        <v>153</v>
+      </c>
+      <c r="B135" s="1">
+        <v>46176</v>
+      </c>
+      <c r="C135" t="s">
+        <v>70</v>
+      </c>
+      <c r="D135" t="s">
+        <v>10</v>
+      </c>
+      <c r="E135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A136" t="s">
+        <v>154</v>
+      </c>
+      <c r="B136" s="1">
+        <v>46177</v>
+      </c>
+      <c r="C136" t="s">
+        <v>60</v>
+      </c>
+      <c r="D136" t="s">
+        <v>15</v>
+      </c>
+      <c r="E136">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A137" t="s">
+        <v>155</v>
+      </c>
+      <c r="B137" s="1">
+        <v>46178</v>
+      </c>
+      <c r="C137" t="s">
+        <v>6</v>
+      </c>
+      <c r="D137" t="s">
+        <v>7</v>
+      </c>
+      <c r="E137">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A138" t="s">
+        <v>156</v>
+      </c>
+      <c r="B138" s="1">
+        <v>46179</v>
+      </c>
+      <c r="C138" t="s">
+        <v>65</v>
+      </c>
+      <c r="D138" t="s">
+        <v>31</v>
+      </c>
+      <c r="E138">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A139" t="s">
+        <v>157</v>
+      </c>
+      <c r="B139" s="1">
+        <v>46180</v>
+      </c>
+      <c r="C139" t="s">
+        <v>12</v>
+      </c>
+      <c r="D139" t="s">
+        <v>17</v>
+      </c>
+      <c r="E139">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A140" t="s">
+        <v>158</v>
+      </c>
+      <c r="B140" s="1">
+        <v>46181</v>
+      </c>
+      <c r="C140" t="s">
+        <v>23</v>
+      </c>
+      <c r="D140" t="s">
+        <v>10</v>
+      </c>
+      <c r="E140">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A141" t="s">
+        <v>159</v>
+      </c>
+      <c r="B141" s="1">
+        <v>46182</v>
+      </c>
+      <c r="C141" t="s">
+        <v>19</v>
+      </c>
+      <c r="D141" t="s">
+        <v>15</v>
+      </c>
+      <c r="E141">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A142" t="s">
+        <v>160</v>
+      </c>
+      <c r="B142" s="1">
+        <v>46183</v>
+      </c>
+      <c r="C142" t="s">
+        <v>42</v>
+      </c>
+      <c r="D142" t="s">
+        <v>7</v>
+      </c>
+      <c r="E142">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A143" t="s">
+        <v>161</v>
+      </c>
+      <c r="B143" s="1">
+        <v>46184</v>
+      </c>
+      <c r="C143" t="s">
+        <v>6</v>
+      </c>
+      <c r="D143" t="s">
+        <v>31</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A144" t="s">
+        <v>162</v>
+      </c>
+      <c r="B144" s="1">
+        <v>46185</v>
+      </c>
+      <c r="C144" t="s">
+        <v>9</v>
+      </c>
+      <c r="D144" t="s">
+        <v>17</v>
+      </c>
+      <c r="E144">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A145" t="s">
+        <v>163</v>
+      </c>
+      <c r="B145" s="1">
+        <v>46186</v>
+      </c>
+      <c r="C145" t="s">
+        <v>70</v>
+      </c>
+      <c r="D145" t="s">
+        <v>10</v>
+      </c>
+      <c r="E145">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A146" t="s">
+        <v>164</v>
+      </c>
+      <c r="B146" s="1">
+        <v>46187</v>
+      </c>
+      <c r="C146" t="s">
+        <v>21</v>
+      </c>
+      <c r="D146" t="s">
+        <v>15</v>
+      </c>
+      <c r="E146">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A147" t="s">
+        <v>165</v>
+      </c>
+      <c r="B147" s="1">
+        <v>46188</v>
+      </c>
+      <c r="C147" t="s">
+        <v>60</v>
+      </c>
+      <c r="D147" t="s">
+        <v>7</v>
+      </c>
+      <c r="E147">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A148" t="s">
+        <v>166</v>
+      </c>
+      <c r="B148" s="1">
+        <v>46189</v>
+      </c>
+      <c r="C148" t="s">
+        <v>12</v>
+      </c>
+      <c r="D148" t="s">
+        <v>31</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A149" t="s">
+        <v>167</v>
+      </c>
+      <c r="B149" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C149" t="s">
+        <v>65</v>
+      </c>
+      <c r="D149" t="s">
+        <v>17</v>
+      </c>
+      <c r="E149">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A150" t="s">
+        <v>168</v>
+      </c>
+      <c r="B150" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C150" t="s">
+        <v>23</v>
+      </c>
+      <c r="D150" t="s">
+        <v>10</v>
+      </c>
+      <c r="E150">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A151" t="s">
+        <v>169</v>
+      </c>
+      <c r="B151" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C151" t="s">
+        <v>19</v>
+      </c>
+      <c r="D151" t="s">
+        <v>15</v>
+      </c>
+      <c r="E151">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A152" t="s">
+        <v>170</v>
+      </c>
+      <c r="B152" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C152" t="s">
+        <v>6</v>
+      </c>
+      <c r="D152" t="s">
+        <v>7</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A153" t="s">
+        <v>171</v>
+      </c>
+      <c r="B153" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C153" t="s">
+        <v>42</v>
+      </c>
+      <c r="D153" t="s">
+        <v>31</v>
+      </c>
+      <c r="E153">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A154" t="s">
+        <v>172</v>
+      </c>
+      <c r="B154" s="1">
+        <v>46195</v>
+      </c>
+      <c r="C154" t="s">
+        <v>9</v>
+      </c>
+      <c r="D154" t="s">
+        <v>17</v>
+      </c>
+      <c r="E154">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A155" t="s">
+        <v>173</v>
+      </c>
+      <c r="B155" s="1">
+        <v>46196</v>
+      </c>
+      <c r="C155" t="s">
+        <v>70</v>
+      </c>
+      <c r="D155" t="s">
+        <v>10</v>
+      </c>
+      <c r="E155">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A156" t="s">
+        <v>174</v>
+      </c>
+      <c r="B156" s="1">
+        <v>46197</v>
+      </c>
+      <c r="C156" t="s">
+        <v>21</v>
+      </c>
+      <c r="D156" t="s">
+        <v>15</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A157" t="s">
+        <v>175</v>
+      </c>
+      <c r="B157" s="1">
+        <v>46198</v>
+      </c>
+      <c r="C157" t="s">
+        <v>60</v>
+      </c>
+      <c r="D157" t="s">
+        <v>7</v>
+      </c>
+      <c r="E157">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A158" t="s">
+        <v>176</v>
+      </c>
+      <c r="B158" s="1">
+        <v>46199</v>
+      </c>
+      <c r="C158" t="s">
+        <v>12</v>
+      </c>
+      <c r="D158" t="s">
+        <v>31</v>
+      </c>
+      <c r="E158">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A159" t="s">
+        <v>177</v>
+      </c>
+      <c r="B159" s="1">
+        <v>46200</v>
+      </c>
+      <c r="C159" t="s">
+        <v>65</v>
+      </c>
+      <c r="D159" t="s">
+        <v>17</v>
+      </c>
+      <c r="E159">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A160" t="s">
+        <v>178</v>
+      </c>
+      <c r="B160" s="1">
+        <v>46201</v>
+      </c>
+      <c r="C160" t="s">
+        <v>23</v>
+      </c>
+      <c r="D160" t="s">
+        <v>10</v>
+      </c>
+      <c r="E160">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A161" t="s">
+        <v>179</v>
+      </c>
+      <c r="B161" s="1">
+        <v>46202</v>
+      </c>
+      <c r="C161" t="s">
+        <v>19</v>
+      </c>
+      <c r="D161" t="s">
+        <v>15</v>
+      </c>
+      <c r="E161">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A162" t="s">
+        <v>180</v>
+      </c>
+      <c r="B162" s="1">
+        <v>46203</v>
+      </c>
+      <c r="C162" t="s">
+        <v>6</v>
+      </c>
+      <c r="D162" t="s">
+        <v>7</v>
+      </c>
+      <c r="E162">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A163" t="s">
+        <v>181</v>
+      </c>
+      <c r="B163" s="1">
+        <v>46204</v>
+      </c>
+      <c r="C163" t="s">
+        <v>42</v>
+      </c>
+      <c r="D163" t="s">
+        <v>31</v>
+      </c>
+      <c r="E163">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A164" t="s">
+        <v>182</v>
+      </c>
+      <c r="B164" s="1">
+        <v>46205</v>
+      </c>
+      <c r="C164" t="s">
+        <v>9</v>
+      </c>
+      <c r="D164" t="s">
+        <v>17</v>
+      </c>
+      <c r="E164">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A165" t="s">
+        <v>183</v>
+      </c>
+      <c r="B165" s="1">
+        <v>46206</v>
+      </c>
+      <c r="C165" t="s">
+        <v>70</v>
+      </c>
+      <c r="D165" t="s">
+        <v>10</v>
+      </c>
+      <c r="E165">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A166" t="s">
+        <v>184</v>
+      </c>
+      <c r="B166" s="1">
+        <v>46207</v>
+      </c>
+      <c r="C166" t="s">
+        <v>21</v>
+      </c>
+      <c r="D166" t="s">
+        <v>15</v>
+      </c>
+      <c r="E166">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A167" t="s">
+        <v>185</v>
+      </c>
+      <c r="B167" s="1">
+        <v>46208</v>
+      </c>
+      <c r="C167" t="s">
+        <v>60</v>
+      </c>
+      <c r="D167" t="s">
+        <v>7</v>
+      </c>
+      <c r="E167">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A168" t="s">
+        <v>186</v>
+      </c>
+      <c r="B168" s="1">
+        <v>46209</v>
+      </c>
+      <c r="C168" t="s">
+        <v>12</v>
+      </c>
+      <c r="D168" t="s">
+        <v>31</v>
+      </c>
+      <c r="E168">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A169" t="s">
+        <v>187</v>
+      </c>
+      <c r="B169" s="1">
+        <v>46210</v>
+      </c>
+      <c r="C169" t="s">
+        <v>65</v>
+      </c>
+      <c r="D169" t="s">
+        <v>17</v>
+      </c>
+      <c r="E169">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A170" t="s">
+        <v>188</v>
+      </c>
+      <c r="B170" s="1">
+        <v>46211</v>
+      </c>
+      <c r="C170" t="s">
+        <v>23</v>
+      </c>
+      <c r="D170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E170">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A171" t="s">
+        <v>189</v>
+      </c>
+      <c r="B171" s="1">
+        <v>46212</v>
+      </c>
+      <c r="C171" t="s">
+        <v>19</v>
+      </c>
+      <c r="D171" t="s">
+        <v>15</v>
+      </c>
+      <c r="E171">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A172" t="s">
+        <v>190</v>
+      </c>
+      <c r="B172" s="1">
+        <v>46213</v>
+      </c>
+      <c r="C172" t="s">
+        <v>6</v>
+      </c>
+      <c r="D172" t="s">
+        <v>7</v>
+      </c>
+      <c r="E172">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A173" t="s">
+        <v>191</v>
+      </c>
+      <c r="B173" s="1">
+        <v>46214</v>
+      </c>
+      <c r="C173" t="s">
+        <v>42</v>
+      </c>
+      <c r="D173" t="s">
+        <v>31</v>
+      </c>
+      <c r="E173">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A174" t="s">
+        <v>192</v>
+      </c>
+      <c r="B174" s="1">
+        <v>46215</v>
+      </c>
+      <c r="C174" t="s">
+        <v>9</v>
+      </c>
+      <c r="D174" t="s">
+        <v>17</v>
+      </c>
+      <c r="E174">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A175" t="s">
+        <v>193</v>
+      </c>
+      <c r="B175" s="1">
+        <v>46216</v>
+      </c>
+      <c r="C175" t="s">
+        <v>70</v>
+      </c>
+      <c r="D175" t="s">
+        <v>10</v>
+      </c>
+      <c r="E175">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A176" t="s">
+        <v>194</v>
+      </c>
+      <c r="B176" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C176" t="s">
+        <v>21</v>
+      </c>
+      <c r="D176" t="s">
+        <v>15</v>
+      </c>
+      <c r="E176">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A177" t="s">
+        <v>195</v>
+      </c>
+      <c r="B177" s="1">
+        <v>46218</v>
+      </c>
+      <c r="C177" t="s">
+        <v>60</v>
+      </c>
+      <c r="D177" t="s">
+        <v>7</v>
+      </c>
+      <c r="E177">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A178" t="s">
+        <v>196</v>
+      </c>
+      <c r="B178" s="1">
+        <v>46219</v>
+      </c>
+      <c r="C178" t="s">
+        <v>12</v>
+      </c>
+      <c r="D178" t="s">
+        <v>31</v>
+      </c>
+      <c r="E178">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A179" t="s">
+        <v>197</v>
+      </c>
+      <c r="B179" s="1">
+        <v>46220</v>
+      </c>
+      <c r="C179" t="s">
+        <v>65</v>
+      </c>
+      <c r="D179" t="s">
+        <v>17</v>
+      </c>
+      <c r="E179">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A180" t="s">
+        <v>198</v>
+      </c>
+      <c r="B180" s="1">
+        <v>46221</v>
+      </c>
+      <c r="C180" t="s">
+        <v>23</v>
+      </c>
+      <c r="D180" t="s">
+        <v>10</v>
+      </c>
+      <c r="E180">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A181" t="s">
+        <v>199</v>
+      </c>
+      <c r="B181" s="1">
+        <v>46222</v>
+      </c>
+      <c r="C181" t="s">
+        <v>19</v>
+      </c>
+      <c r="D181" t="s">
+        <v>15</v>
+      </c>
+      <c r="E181">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A182" t="s">
+        <v>200</v>
+      </c>
+      <c r="B182" s="1">
+        <v>46223</v>
+      </c>
+      <c r="C182" t="s">
+        <v>6</v>
+      </c>
+      <c r="D182" t="s">
+        <v>7</v>
+      </c>
+      <c r="E182">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A183" t="s">
+        <v>201</v>
+      </c>
+      <c r="B183" s="1">
+        <v>46224</v>
+      </c>
+      <c r="C183" t="s">
+        <v>42</v>
+      </c>
+      <c r="D183" t="s">
+        <v>31</v>
+      </c>
+      <c r="E183">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A184" t="s">
+        <v>202</v>
+      </c>
+      <c r="B184" s="1">
+        <v>46225</v>
+      </c>
+      <c r="C184" t="s">
+        <v>9</v>
+      </c>
+      <c r="D184" t="s">
+        <v>17</v>
+      </c>
+      <c r="E184">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A185" t="s">
+        <v>203</v>
+      </c>
+      <c r="B185" s="1">
+        <v>46226</v>
+      </c>
+      <c r="C185" t="s">
+        <v>70</v>
+      </c>
+      <c r="D185" t="s">
+        <v>10</v>
+      </c>
+      <c r="E185">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A186" t="s">
+        <v>204</v>
+      </c>
+      <c r="B186" s="1">
+        <v>46227</v>
+      </c>
+      <c r="C186" t="s">
+        <v>21</v>
+      </c>
+      <c r="D186" t="s">
+        <v>15</v>
+      </c>
+      <c r="E186">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A187" t="s">
+        <v>205</v>
+      </c>
+      <c r="B187" s="1">
+        <v>46228</v>
+      </c>
+      <c r="C187" t="s">
+        <v>60</v>
+      </c>
+      <c r="D187" t="s">
+        <v>7</v>
+      </c>
+      <c r="E187">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A188" t="s">
+        <v>206</v>
+      </c>
+      <c r="B188" s="1">
+        <v>46229</v>
+      </c>
+      <c r="C188" t="s">
+        <v>12</v>
+      </c>
+      <c r="D188" t="s">
+        <v>31</v>
+      </c>
+      <c r="E188">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A189" t="s">
+        <v>207</v>
+      </c>
+      <c r="B189" s="1">
+        <v>46230</v>
+      </c>
+      <c r="C189" t="s">
+        <v>65</v>
+      </c>
+      <c r="D189" t="s">
+        <v>17</v>
+      </c>
+      <c r="E189">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A190" t="s">
+        <v>208</v>
+      </c>
+      <c r="B190" s="1">
+        <v>46231</v>
+      </c>
+      <c r="C190" t="s">
+        <v>23</v>
+      </c>
+      <c r="D190" t="s">
+        <v>10</v>
+      </c>
+      <c r="E190">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A191" t="s">
+        <v>209</v>
+      </c>
+      <c r="B191" s="1">
+        <v>46232</v>
+      </c>
+      <c r="C191" t="s">
+        <v>19</v>
+      </c>
+      <c r="D191" t="s">
+        <v>15</v>
+      </c>
+      <c r="E191">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A192" t="s">
+        <v>210</v>
+      </c>
+      <c r="B192" s="1">
+        <v>46233</v>
+      </c>
+      <c r="C192" t="s">
+        <v>6</v>
+      </c>
+      <c r="D192" t="s">
+        <v>7</v>
+      </c>
+      <c r="E192">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A193" t="s">
+        <v>211</v>
+      </c>
+      <c r="B193" s="1">
+        <v>46234</v>
+      </c>
+      <c r="C193" t="s">
+        <v>42</v>
+      </c>
+      <c r="D193" t="s">
+        <v>31</v>
+      </c>
+      <c r="E193">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A194" t="s">
+        <v>212</v>
+      </c>
+      <c r="B194" s="1">
+        <v>46235</v>
+      </c>
+      <c r="C194" t="s">
+        <v>9</v>
+      </c>
+      <c r="D194" t="s">
+        <v>17</v>
+      </c>
+      <c r="E194">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A195" t="s">
+        <v>213</v>
+      </c>
+      <c r="B195" s="1">
+        <v>46236</v>
+      </c>
+      <c r="C195" t="s">
+        <v>70</v>
+      </c>
+      <c r="D195" t="s">
+        <v>10</v>
+      </c>
+      <c r="E195">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A196" t="s">
+        <v>214</v>
+      </c>
+      <c r="B196" s="1">
+        <v>46237</v>
+      </c>
+      <c r="C196" t="s">
+        <v>21</v>
+      </c>
+      <c r="D196" t="s">
+        <v>15</v>
+      </c>
+      <c r="E196">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A197" t="s">
+        <v>215</v>
+      </c>
+      <c r="B197" s="1">
+        <v>46238</v>
+      </c>
+      <c r="C197" t="s">
+        <v>60</v>
+      </c>
+      <c r="D197" t="s">
+        <v>7</v>
+      </c>
+      <c r="E197">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A198" t="s">
+        <v>216</v>
+      </c>
+      <c r="B198" s="1">
+        <v>46239</v>
+      </c>
+      <c r="C198" t="s">
+        <v>12</v>
+      </c>
+      <c r="D198" t="s">
+        <v>31</v>
+      </c>
+      <c r="E198">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A199" t="s">
+        <v>217</v>
+      </c>
+      <c r="B199" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C199" t="s">
+        <v>65</v>
+      </c>
+      <c r="D199" t="s">
+        <v>17</v>
+      </c>
+      <c r="E199">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A200" t="s">
+        <v>218</v>
+      </c>
+      <c r="B200" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C200" t="s">
+        <v>23</v>
+      </c>
+      <c r="D200" t="s">
+        <v>10</v>
+      </c>
+      <c r="E200">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A201" t="s">
+        <v>219</v>
+      </c>
+      <c r="B201" s="1">
+        <v>46242</v>
+      </c>
+      <c r="C201" t="s">
+        <v>19</v>
+      </c>
+      <c r="D201" t="s">
+        <v>15</v>
+      </c>
+      <c r="E201">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>